<commit_message>
Adding measurement results EXCE:
</commit_message>
<xml_diff>
--- a/EXCEL FILEOVI/ZAVRSNI RESULTS - MJERENJA.xlsx
+++ b/EXCEL FILEOVI/ZAVRSNI RESULTS - MJERENJA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/523341e057c2d1b5/Documents/2526 - LJETNI SEMESTAR/Bachelor-Thesis/EXCEL FILEOVI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{A8C83972-76C5-4A6B-842F-923ACDC1EACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{156EC5CC-E0B4-4264-8753-AE6F2818634E}"/>
+  <xr:revisionPtr revIDLastSave="239" documentId="8_{A8C83972-76C5-4A6B-842F-923ACDC1EACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B59EFB5-DCBB-4B73-88A3-00B94E509625}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{84FF4933-D298-41E7-88E7-BD26EEEC429A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{84FF4933-D298-41E7-88E7-BD26EEEC429A}"/>
   </bookViews>
   <sheets>
     <sheet name="SZC" sheetId="1" r:id="rId1"/>
@@ -158,13 +158,13 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -180,6 +180,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -529,904 +533,904 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="F1" s="1" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="F1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="K1" s="1" t="s">
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="K1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="P1" s="1" t="s">
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="P1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="U1" s="1" t="s">
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="U1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="Q2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="S2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="U2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="V2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="2" t="s">
+      <c r="W2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="X2" s="2" t="s">
+      <c r="X2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>4.0629999999999997</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <f>10^(B3/20)</f>
         <v>1.5964304395662618</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f>C3^2</f>
         <v>2.5485901483737279</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>1</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="2">
         <v>7.0910000000000002</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="2">
         <f>10^(G3/20)</f>
         <v>2.2622989815726413</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="2">
         <f>H3^2</f>
         <v>5.1179966820246099</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="2">
         <v>9.6829999999999998</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="2">
         <f>10^(L3/20)</f>
         <v>3.0489478770799572</v>
       </c>
-      <c r="N3" s="3">
+      <c r="N3" s="2">
         <f>M3^2</f>
         <v>9.2960831571503775</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>1</v>
       </c>
-      <c r="Q3" s="3">
+      <c r="Q3" s="2">
         <v>10.382999999999999</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="2">
         <f>10^(Q3/20)</f>
         <v>3.3048366634147781</v>
       </c>
-      <c r="S3" s="3">
+      <c r="S3" s="2">
         <f>R3^2</f>
         <v>10.921945371850523</v>
       </c>
-      <c r="U3" s="2">
+      <c r="U3" s="1">
         <v>1</v>
       </c>
-      <c r="V3" s="3">
+      <c r="V3" s="2">
         <v>10.859</v>
       </c>
-      <c r="W3" s="3">
+      <c r="W3" s="2">
         <f>10^(V3/20)</f>
         <v>3.491001215280912</v>
       </c>
-      <c r="X3" s="3">
+      <c r="X3" s="2">
         <f>W3^2</f>
         <v>12.187089485092805</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>-1.0629999999999999</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <f t="shared" ref="C4:C10" si="0">10^(B4/20)</f>
         <v>0.88480995451736077</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f t="shared" ref="D4:D10" si="1">C4^2</f>
         <v>0.78288865561301402</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>2</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>-0.498</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <f t="shared" ref="H4:H10" si="2">10^(G4/20)</f>
         <v>0.94427827936447872</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="2">
         <f t="shared" ref="I4:I10" si="3">H4^2</f>
         <v>0.89166146887954056</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>2</v>
       </c>
-      <c r="L4" s="3">
+      <c r="L4" s="2">
         <v>-0.90400000000000003</v>
       </c>
-      <c r="M4" s="3">
+      <c r="M4" s="2">
         <f t="shared" ref="M4:M10" si="4">10^(L4/20)</f>
         <v>0.90115604433970453</v>
       </c>
-      <c r="N4" s="3">
+      <c r="N4" s="2">
         <f t="shared" ref="N4:N10" si="5">M4^2</f>
         <v>0.81208221624998356</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>2</v>
       </c>
-      <c r="Q4" s="3">
+      <c r="Q4" s="2">
         <v>-1.488</v>
       </c>
-      <c r="R4" s="3">
+      <c r="R4" s="2">
         <f t="shared" ref="R4:R10" si="6">10^(Q4/20)</f>
         <v>0.84255837533982603</v>
       </c>
-      <c r="S4" s="3">
+      <c r="S4" s="2">
         <f t="shared" ref="S4:S10" si="7">R4^2</f>
         <v>0.70990461585528719</v>
       </c>
-      <c r="U4" s="2">
+      <c r="U4" s="1">
         <v>2</v>
       </c>
-      <c r="V4" s="3">
+      <c r="V4" s="2">
         <v>-2.0630000000000002</v>
       </c>
-      <c r="W4" s="3">
+      <c r="W4" s="2">
         <f t="shared" ref="W4:W10" si="8">10^(V4/20)</f>
         <v>0.78858770203367434</v>
       </c>
-      <c r="X4" s="3">
+      <c r="X4" s="2">
         <f t="shared" ref="X4:X10" si="9">W4^2</f>
         <v>0.62187056379875116</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>-12.91</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <f t="shared" si="0"/>
         <v>0.22620385397696208</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <f t="shared" si="1"/>
         <v>5.1168183554030786E-2</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <v>-11.615</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="2">
         <f t="shared" si="2"/>
         <v>0.26257295998844254</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="2">
         <f t="shared" si="3"/>
         <v>6.8944559317092244E-2</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>3</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="2">
         <v>-11.195</v>
       </c>
-      <c r="M5" s="3">
+      <c r="M5" s="2">
         <f t="shared" si="4"/>
         <v>0.27558146212469903</v>
       </c>
-      <c r="N5" s="3">
+      <c r="N5" s="2">
         <f t="shared" si="5"/>
         <v>7.5945142266786919E-2</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>3</v>
       </c>
-      <c r="Q5" s="3">
+      <c r="Q5" s="2">
         <v>-13.353</v>
       </c>
-      <c r="R5" s="3">
+      <c r="R5" s="2">
         <f t="shared" si="6"/>
         <v>0.2149562118658318</v>
       </c>
-      <c r="S5" s="3">
+      <c r="S5" s="2">
         <f t="shared" si="7"/>
         <v>4.620617301970837E-2</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>3</v>
       </c>
-      <c r="V5" s="3">
+      <c r="V5" s="2">
         <v>-15.952</v>
       </c>
-      <c r="W5" s="3">
+      <c r="W5" s="2">
         <f t="shared" si="8"/>
         <v>0.15936758810287666</v>
       </c>
-      <c r="X5" s="3">
+      <c r="X5" s="2">
         <f t="shared" si="9"/>
         <v>2.5398028137728151E-2</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>-15.875</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <f t="shared" si="0"/>
         <v>0.16078665490525609</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <f t="shared" si="1"/>
         <v>2.5852348395621914E-2</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>4</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <v>-17.678000000000001</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="2">
         <f t="shared" si="2"/>
         <v>0.13064716797220155</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="2">
         <f t="shared" si="3"/>
         <v>1.7068682499156645E-2</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>4</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L6" s="2">
         <v>-18.815000000000001</v>
       </c>
-      <c r="M6" s="3">
+      <c r="M6" s="2">
         <f t="shared" si="4"/>
         <v>0.11461725415311876</v>
       </c>
-      <c r="N6" s="3">
+      <c r="N6" s="2">
         <f t="shared" si="5"/>
         <v>1.3137114949600619E-2</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>4</v>
       </c>
-      <c r="Q6" s="3">
+      <c r="Q6" s="2">
         <v>-17.846</v>
       </c>
-      <c r="R6" s="3">
+      <c r="R6" s="2">
         <f t="shared" si="6"/>
         <v>0.12814450859457868</v>
       </c>
-      <c r="S6" s="3">
+      <c r="S6" s="2">
         <f t="shared" si="7"/>
         <v>1.642101508294605E-2</v>
       </c>
-      <c r="U6" s="2">
+      <c r="U6" s="1">
         <v>4</v>
       </c>
-      <c r="V6" s="3">
+      <c r="V6" s="2">
         <v>-18.533999999999999</v>
       </c>
-      <c r="W6" s="3">
+      <c r="W6" s="2">
         <f t="shared" si="8"/>
         <v>0.11838590542018096</v>
       </c>
-      <c r="X6" s="3">
+      <c r="X6" s="2">
         <f t="shared" si="9"/>
         <v>1.4015222602156031E-2</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>-22.629000000000001</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <f t="shared" si="0"/>
         <v>7.3883932011749143E-2</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <f t="shared" si="1"/>
         <v>5.4588354095167699E-3</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>5</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <v>-20.309999999999999</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="2">
         <f t="shared" si="2"/>
         <v>9.6493931180558212E-2</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="2">
         <f t="shared" si="3"/>
         <v>9.3110787546783046E-3</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>5</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L7" s="2">
         <v>-26.321000000000002</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M7" s="2">
         <f t="shared" si="4"/>
         <v>4.8300319104122941E-2</v>
       </c>
-      <c r="N7" s="3">
+      <c r="N7" s="2">
         <f t="shared" si="5"/>
         <v>2.3329208255601034E-3</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>5</v>
       </c>
-      <c r="Q7" s="3">
+      <c r="Q7" s="2">
         <v>-28.152999999999999</v>
       </c>
-      <c r="R7" s="3">
+      <c r="R7" s="2">
         <f t="shared" si="6"/>
         <v>3.9115600329580377E-2</v>
       </c>
-      <c r="S7" s="3">
+      <c r="S7" s="2">
         <f t="shared" si="7"/>
         <v>1.5300301891434686E-3</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>5</v>
       </c>
-      <c r="V7" s="3">
+      <c r="V7" s="2">
         <v>-24.494</v>
       </c>
-      <c r="W7" s="3">
+      <c r="W7" s="2">
         <f t="shared" si="8"/>
         <v>5.960737545096844E-2</v>
       </c>
-      <c r="X7" s="3">
+      <c r="X7" s="2">
         <f t="shared" si="9"/>
         <v>3.5530392081527151E-3</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>-23.977</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <f t="shared" si="0"/>
         <v>6.3263031641686535E-2</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <f t="shared" si="1"/>
         <v>4.0022111724970317E-3</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>6</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="2">
         <v>-28.501999999999999</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="2">
         <f t="shared" si="2"/>
         <v>3.7575087449048715E-2</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="2">
         <f t="shared" si="3"/>
         <v>1.4118871968036583E-3</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>6</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L8" s="2">
         <v>-24.355</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M8" s="2">
         <f t="shared" si="4"/>
         <v>6.0568943728724685E-2</v>
       </c>
-      <c r="N8" s="3">
+      <c r="N8" s="2">
         <f t="shared" si="5"/>
         <v>3.6685969444134174E-3</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>6</v>
       </c>
-      <c r="Q8" s="3">
+      <c r="Q8" s="2">
         <v>-29.902999999999999</v>
       </c>
-      <c r="R8" s="3">
+      <c r="R8" s="2">
         <f t="shared" si="6"/>
         <v>3.1977904412428169E-2</v>
       </c>
-      <c r="S8" s="3">
+      <c r="S8" s="2">
         <f t="shared" si="7"/>
         <v>1.0225863706103931E-3</v>
       </c>
-      <c r="U8" s="2">
+      <c r="U8" s="1">
         <v>6</v>
       </c>
-      <c r="V8" s="3">
+      <c r="V8" s="2">
         <v>-31.516999999999999</v>
       </c>
-      <c r="W8" s="3">
+      <c r="W8" s="2">
         <f t="shared" si="8"/>
         <v>2.6555225886105299E-2</v>
       </c>
-      <c r="X8" s="3">
+      <c r="X8" s="2">
         <f t="shared" si="9"/>
         <v>7.0518002186207695E-4</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>-29.119</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <f t="shared" si="0"/>
         <v>3.4998545827391141E-2</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <f t="shared" si="1"/>
         <v>1.2248982100319977E-3</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>7</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="2">
         <v>-25.485800000000001</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="2">
         <f t="shared" si="2"/>
         <v>5.3175306275293328E-2</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="2">
         <f t="shared" si="3"/>
         <v>2.8276131974712499E-3</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>7</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L9" s="2">
         <v>-28.395</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="2">
         <f t="shared" si="4"/>
         <v>3.8040831393319027E-2</v>
       </c>
-      <c r="N9" s="3">
+      <c r="N9" s="2">
         <f t="shared" si="5"/>
         <v>1.4471048530949264E-3</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>7</v>
       </c>
-      <c r="Q9" s="3">
+      <c r="Q9" s="2">
         <v>-28.931999999999999</v>
       </c>
-      <c r="R9" s="3">
+      <c r="R9" s="2">
         <f t="shared" si="6"/>
         <v>3.5760205018090234E-2</v>
       </c>
-      <c r="S9" s="3">
+      <c r="S9" s="2">
         <f t="shared" si="7"/>
         <v>1.278792262935846E-3</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>7</v>
       </c>
-      <c r="V9" s="3">
+      <c r="V9" s="2">
         <v>-37.713000000000001</v>
       </c>
-      <c r="W9" s="3">
+      <c r="W9" s="2">
         <f t="shared" si="8"/>
         <v>1.3012178132465021E-2</v>
       </c>
-      <c r="X9" s="3">
+      <c r="X9" s="2">
         <f t="shared" si="9"/>
         <v>1.6931677975100089E-4</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>-27.27</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <f t="shared" si="0"/>
         <v>4.3301206773800408E-2</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <f t="shared" si="1"/>
         <v>1.8749945080674183E-3</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>8</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="2">
         <v>-32.256999999999998</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="2">
         <f t="shared" si="2"/>
         <v>2.4386529538195086E-2</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="2">
         <f t="shared" si="3"/>
         <v>5.9470282291726147E-4</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>8</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L10" s="2">
         <v>-38.296999999999997</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M10" s="2">
         <f t="shared" si="4"/>
         <v>1.2166061289590899E-2</v>
       </c>
-      <c r="N10" s="3">
+      <c r="N10" s="2">
         <f t="shared" si="5"/>
         <v>1.4801304730208215E-4</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>8</v>
       </c>
-      <c r="Q10" s="3">
+      <c r="Q10" s="2">
         <v>-32.042999999999999</v>
       </c>
-      <c r="R10" s="3">
+      <c r="R10" s="2">
         <f t="shared" si="6"/>
         <v>2.4994819221221688E-2</v>
       </c>
-      <c r="S10" s="3">
+      <c r="S10" s="2">
         <f t="shared" si="7"/>
         <v>6.2474098790155314E-4</v>
       </c>
-      <c r="U10" s="2">
+      <c r="U10" s="1">
         <v>8</v>
       </c>
-      <c r="V10" s="3">
+      <c r="V10" s="2">
         <v>-33.606999999999999</v>
       </c>
-      <c r="W10" s="3">
+      <c r="W10" s="2">
         <f t="shared" si="8"/>
         <v>2.0876130354084546E-2</v>
       </c>
-      <c r="X10" s="3">
+      <c r="X10" s="2">
         <f t="shared" si="9"/>
         <v>4.3581281856073015E-4</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <f>SQRT(SUM(D4:D10)/D3)</f>
         <v>0.58509351275376109</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="F11" s="2" t="s">
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="F11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="2">
         <f>SQRT(SUM(I4:I10)/I3)</f>
         <v>0.44021661415927188</v>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="K11" s="2" t="s">
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="K11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="2">
         <f>SQRT(SUM(N4:N10)/N3)</f>
         <v>0.31266183071490777</v>
       </c>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="P11" s="2" t="s">
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="P11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="Q11" s="3">
+      <c r="Q11" s="2">
         <f>SQRT(SUM(S4:S10)/S3)</f>
         <v>0.26672095828047437</v>
       </c>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="U11" s="2" t="s">
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
+      <c r="U11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="V11" s="3">
+      <c r="V11" s="2">
         <f>SQRT(SUM(X4:X10)/X3)</f>
         <v>0.23379493133774276</v>
       </c>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
+      <c r="W11" s="1"/>
+      <c r="X11" s="1"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <f>B11*100</f>
         <v>58.509351275376112</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="F12" s="4" t="s">
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="F12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <f>G11*100</f>
         <v>44.021661415927191</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="K12" s="4" t="s">
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="K12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L12" s="4">
         <f>L11*100</f>
         <v>31.266183071490776</v>
       </c>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="P12" s="4" t="s">
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="P12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="Q12" s="5">
+      <c r="Q12" s="4">
         <f>Q11*100</f>
         <v>26.672095828047439</v>
       </c>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
-      <c r="U12" s="4" t="s">
+      <c r="R12" s="1"/>
+      <c r="S12" s="1"/>
+      <c r="U12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="V12" s="5">
+      <c r="V12" s="4">
         <f>V11*100</f>
         <v>23.379493133774275</v>
       </c>
-      <c r="W12" s="2"/>
-      <c r="X12" s="2"/>
+      <c r="W12" s="1"/>
+      <c r="X12" s="1"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <f>(B16^2/250) * 1000</f>
         <v>12.67502404</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="F13" s="2" t="s">
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="F13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <f>(G16^2/500) * 1000</f>
         <v>12.490002</v>
       </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="K13" s="2" t="s">
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="K13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L13" s="2">
+      <c r="L13" s="1">
         <f>(L16^2/1000) * 1000</f>
         <v>10.864275210000001</v>
       </c>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="P13" s="2" t="s">
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="P13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <f>(Q16^2/1500) * 1000</f>
         <v>8.3983536599999997</v>
       </c>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="U13" s="2" t="s">
+      <c r="R13" s="1"/>
+      <c r="S13" s="1"/>
+      <c r="U13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="1">
         <f>(V16^2/2000) * 1000</f>
         <v>6.9788480000000011</v>
       </c>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
+      <c r="W13" s="1"/>
+      <c r="X13" s="1"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>116.68</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="F14" s="2" t="s">
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="F14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>116.68</v>
       </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="K14" s="2" t="s">
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="K14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L14" s="2">
+      <c r="L14" s="1">
         <v>116.68</v>
       </c>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="P14" s="2" t="s">
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="P14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>116.68</v>
       </c>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="U14" s="2" t="s">
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="U14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="1">
         <v>116.68</v>
       </c>
-      <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
+      <c r="W14" s="1"/>
+      <c r="X14" s="1"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <f>(B13/B14)*100</f>
         <v>10.863064826876927</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="F15" s="4" t="s">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="F15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <f>(G16^2/500) * 1000</f>
         <v>12.490002</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="K15" s="4" t="s">
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="K15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L15" s="4">
+      <c r="L15" s="3">
         <f>(L13/L14)*100</f>
         <v>9.3111717603702431</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="P15" s="4" t="s">
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="P15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="Q15" s="4">
+      <c r="Q15" s="3">
         <f>(Q13/Q14)*100</f>
         <v>7.1977662495714769</v>
       </c>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-      <c r="U15" s="4" t="s">
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="U15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="V15" s="4">
+      <c r="V15" s="3">
         <f>(V13/V14)*100</f>
         <v>5.9811861501542687</v>
       </c>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
+      <c r="W15" s="1"/>
+      <c r="X15" s="1"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.45">
       <c r="B16">
@@ -1477,508 +1481,553 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="F1" s="1" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="F1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="K1" s="1" t="s">
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="K1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3">
+      <c r="B3" s="2">
+        <v>6.5670000000000002</v>
+      </c>
+      <c r="C3" s="2">
         <f>10^(B3/20)</f>
+        <v>2.1298548146980401</v>
+      </c>
+      <c r="D3" s="2">
+        <f>C3^2</f>
+        <v>4.5362815316924223</v>
+      </c>
+      <c r="F3" s="1">
         <v>1</v>
       </c>
-      <c r="D3" s="3">
-        <f>C3^2</f>
+      <c r="G3" s="2">
+        <v>10.045999999999999</v>
+      </c>
+      <c r="H3" s="2">
+        <f>10^(G3/20)</f>
+        <v>3.1790693356433639</v>
+      </c>
+      <c r="I3" s="2">
+        <f>H3^2</f>
+        <v>10.106481840827939</v>
+      </c>
+      <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="F3" s="2">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3">
-        <f>10^(G3/20)</f>
-        <v>1</v>
-      </c>
-      <c r="I3" s="3">
-        <f>H3^2</f>
-        <v>1</v>
-      </c>
-      <c r="K3" s="2">
-        <v>1</v>
-      </c>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3">
+      <c r="L3" s="2">
+        <v>14.49</v>
+      </c>
+      <c r="M3" s="2">
         <f>10^(L3/20)</f>
-        <v>1</v>
-      </c>
-      <c r="N3" s="3">
+        <v>5.3027359262921454</v>
+      </c>
+      <c r="N3" s="2">
         <f>M3^2</f>
-        <v>1</v>
+        <v>28.119008303989418</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3">
+      <c r="B4" s="2">
+        <v>-21.466000000000001</v>
+      </c>
+      <c r="C4" s="2">
         <f t="shared" ref="C4:C10" si="0">10^(B4/20)</f>
-        <v>1</v>
-      </c>
-      <c r="D4" s="3">
+        <v>8.4469514884457822E-2</v>
+      </c>
+      <c r="D4" s="2">
         <f t="shared" ref="D4:D10" si="1">C4^2</f>
-        <v>1</v>
-      </c>
-      <c r="F4" s="2">
+        <v>7.1350989448156418E-3</v>
+      </c>
+      <c r="F4" s="1">
         <v>2</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3">
+      <c r="G4" s="2">
+        <v>-5.1109999999999998</v>
+      </c>
+      <c r="H4" s="2">
         <f t="shared" ref="H4:H10" si="2">10^(G4/20)</f>
-        <v>1</v>
-      </c>
-      <c r="I4" s="3">
+        <v>0.5552006935978655</v>
+      </c>
+      <c r="I4" s="2">
         <f t="shared" ref="I4:I10" si="3">H4^2</f>
-        <v>1</v>
-      </c>
-      <c r="K4" s="2">
+        <v>0.30824781017155095</v>
+      </c>
+      <c r="K4" s="1">
         <v>2</v>
       </c>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3">
+      <c r="L4" s="2">
+        <v>-0.28699999999999998</v>
+      </c>
+      <c r="M4" s="2">
         <f t="shared" ref="M4:M10" si="4">10^(L4/20)</f>
-        <v>1</v>
-      </c>
-      <c r="N4" s="3">
+        <v>0.96749783086137087</v>
+      </c>
+      <c r="N4" s="2">
         <f t="shared" ref="N4:N10" si="5">M4^2</f>
-        <v>1</v>
+        <v>0.93605205272145775</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3">
+      <c r="B5" s="2">
+        <v>-57.890999999999998</v>
+      </c>
+      <c r="C5" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D5" s="3">
+        <v>1.2748233220357839E-3</v>
+      </c>
+      <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F5" s="2">
+        <v>1.6251745024063519E-6</v>
+      </c>
+      <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3">
+      <c r="G5" s="2">
+        <v>-33.796999999999997</v>
+      </c>
+      <c r="H5" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I5" s="3">
+        <v>2.0424432577690541E-2</v>
+      </c>
+      <c r="I5" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K5" s="2">
+        <v>4.1715744612062664E-4</v>
+      </c>
+      <c r="K5" s="1">
         <v>3</v>
       </c>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3">
+      <c r="L5" s="2">
+        <v>-32.042000000000002</v>
+      </c>
+      <c r="M5" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N5" s="3">
+        <v>2.499769702178507E-2</v>
+      </c>
+      <c r="N5" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>6.2488485639296211E-4</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3">
+      <c r="B6" s="2">
+        <v>-58.859000000000002</v>
+      </c>
+      <c r="C6" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D6" s="3">
+        <v>1.1403810712264746E-3</v>
+      </c>
+      <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F6" s="2">
+        <v>1.3004689876116418E-6</v>
+      </c>
+      <c r="F6" s="1">
         <v>4</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3">
+      <c r="G6" s="2">
+        <v>-46.024000000000001</v>
+      </c>
+      <c r="H6" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I6" s="3">
+        <v>4.9980431357823868E-3</v>
+      </c>
+      <c r="I6" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K6" s="2">
+        <v>2.4980435187141435E-5</v>
+      </c>
+      <c r="K6" s="1">
         <v>4</v>
       </c>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3">
+      <c r="L6" s="2">
+        <v>-38.003</v>
+      </c>
+      <c r="M6" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N6" s="3">
+        <v>1.2584906694428742E-2</v>
+      </c>
+      <c r="N6" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>1.5837987650747735E-4</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3">
+      <c r="B7" s="2">
+        <v>-60.436</v>
+      </c>
+      <c r="C7" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D7" s="3">
+        <v>9.5104266415739231E-4</v>
+      </c>
+      <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F7" s="2">
+        <v>9.0448214904759046E-7</v>
+      </c>
+      <c r="F7" s="1">
         <v>5</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3">
+      <c r="G7" s="2">
+        <v>-43.34</v>
+      </c>
+      <c r="H7" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I7" s="3">
+        <v>6.8076935869374067E-3</v>
+      </c>
+      <c r="I7" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K7" s="2">
+        <v>4.6344691973628695E-5</v>
+      </c>
+      <c r="K7" s="1">
         <v>5</v>
       </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3">
+      <c r="L7" s="2">
+        <v>-30.152000000000001</v>
+      </c>
+      <c r="M7" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N7" s="3">
+        <v>3.1074203103885853E-2</v>
+      </c>
+      <c r="N7" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>9.656060985415492E-4</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3">
+      <c r="B8" s="2">
+        <v>-65.933999999999997</v>
+      </c>
+      <c r="C8" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D8" s="3">
+        <v>5.0501002567031631E-4</v>
+      </c>
+      <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F8" s="2">
+        <v>2.5503512602753353E-7</v>
+      </c>
+      <c r="F8" s="1">
         <v>6</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3">
+      <c r="G8" s="2">
+        <v>-48.472999999999999</v>
+      </c>
+      <c r="H8" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I8" s="3">
+        <v>3.7700750874124912E-3</v>
+      </c>
+      <c r="I8" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K8" s="2">
+        <v>1.4213466164728304E-5</v>
+      </c>
+      <c r="K8" s="1">
         <v>6</v>
       </c>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3">
+      <c r="L8" s="2">
+        <v>-41.411000000000001</v>
+      </c>
+      <c r="M8" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N8" s="3">
+        <v>8.5006082068485832E-3</v>
+      </c>
+      <c r="N8" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>7.2260339886341486E-5</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3">
+      <c r="B9" s="2">
+        <v>-57.265999999999998</v>
+      </c>
+      <c r="C9" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D9" s="3">
+        <v>1.369935121586242E-3</v>
+      </c>
+      <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F9" s="2">
+        <v>1.8767222373555116E-6</v>
+      </c>
+      <c r="F9" s="1">
         <v>7</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3">
+      <c r="G9" s="2">
+        <v>-38.488999999999997</v>
+      </c>
+      <c r="H9" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I9" s="3">
+        <v>1.1900083260453193E-2</v>
+      </c>
+      <c r="I9" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K9" s="2">
+        <v>1.416119816057183E-4</v>
+      </c>
+      <c r="K9" s="1">
         <v>7</v>
       </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3">
+      <c r="L9" s="2">
+        <v>-33.200000000000003</v>
+      </c>
+      <c r="M9" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N9" s="3">
+        <v>2.1877616239495513E-2</v>
+      </c>
+      <c r="N9" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>4.7863009232263778E-4</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3">
+      <c r="B10" s="2">
+        <v>-71.540999999999997</v>
+      </c>
+      <c r="C10" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D10" s="3">
+        <v>2.6481952363117267E-4</v>
+      </c>
+      <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F10" s="2">
+        <v>7.0129380096241214E-8</v>
+      </c>
+      <c r="F10" s="1">
         <v>8</v>
       </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3">
+      <c r="G10" s="2">
+        <v>-53.252000000000002</v>
+      </c>
+      <c r="H10" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I10" s="3">
+        <v>2.1747032324403496E-3</v>
+      </c>
+      <c r="I10" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K10" s="2">
+        <v>4.7293341491865055E-6</v>
+      </c>
+      <c r="K10" s="1">
         <v>8</v>
       </c>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3">
+      <c r="L10" s="2">
+        <v>-44.701000000000001</v>
+      </c>
+      <c r="M10" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N10" s="3">
+        <v>5.8203620451894667E-3</v>
+      </c>
+      <c r="N10" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>3.3876614337082113E-5</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <f>SQRT(SUM(D4:D10)/D3)</f>
-        <v>2.6457513110645907</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="F11" s="2" t="s">
+        <v>3.9676513169133773E-2</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="F11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="2">
         <f>SQRT(SUM(I4:I10)/I3)</f>
-        <v>2.6457513110645907</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="K11" s="2" t="s">
+        <v>0.17482628861983959</v>
+      </c>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="K11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="2">
         <f>SQRT(SUM(N4:N10)/N3)</f>
-        <v>2.6457513110645907</v>
-      </c>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
+        <v>0.18267986765764549</v>
+      </c>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <f>B11*100</f>
-        <v>264.57513110645908</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="F12" s="4" t="s">
+        <v>3.9676513169133774</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="F12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <f>G11*100</f>
-        <v>264.57513110645908</v>
-      </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="K12" s="4" t="s">
+        <v>17.482628861983958</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="K12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L12" s="4">
         <f>L11*100</f>
-        <v>264.57513110645908</v>
-      </c>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
+        <v>18.267986765764547</v>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="2">
-        <f>(B16^2/250) * 1000</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="F13" s="2" t="s">
+      <c r="B13" s="1">
+        <v>2.8130000000000002</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="F13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="2">
-        <f>(G16^2/250) * 1000</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="K13" s="2" t="s">
+      <c r="G13" s="1">
+        <v>76.05</v>
+      </c>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="K13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L13" s="2">
-        <f>(L16^2/250) * 1000</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
+      <c r="L13" s="1">
+        <v>208.01300000000001</v>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="2">
-        <v>116.68</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="F14" s="2" t="s">
+      <c r="B14" s="1">
+        <v>71.62</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="F14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G14" s="2">
-        <v>116.68</v>
-      </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="K14" s="2" t="s">
+      <c r="G14" s="1">
+        <v>372.423</v>
+      </c>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="K14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L14" s="2">
-        <v>116.68</v>
-      </c>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
+      <c r="L14" s="1">
+        <v>615.92999999999995</v>
+      </c>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <f>(B13/B14)*100</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="F15" s="4" t="s">
+        <v>3.9276738341245463</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="F15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <f>(G13/G14)*100</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="K15" s="4" t="s">
+        <v>20.420328497434369</v>
+      </c>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="K15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L15" s="4">
+      <c r="L15" s="3">
         <f>(L13/L14)*100</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
+        <v>33.772181903787775</v>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2010,508 +2059,553 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="F1" s="1" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="F1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="K1" s="1" t="s">
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="K1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3">
+      <c r="B3" s="2">
+        <v>-5.9939999999999998</v>
+      </c>
+      <c r="C3" s="2">
         <f>10^(B3/20)</f>
+        <v>0.50153356110665925</v>
+      </c>
+      <c r="D3" s="2">
+        <f>C3^2</f>
+        <v>0.2515359129163271</v>
+      </c>
+      <c r="F3" s="1">
         <v>1</v>
       </c>
-      <c r="D3" s="3">
-        <f>C3^2</f>
+      <c r="G3" s="2">
+        <v>10.06</v>
+      </c>
+      <c r="H3" s="2">
+        <f>10^(G3/20)</f>
+        <v>3.1841975217261251</v>
+      </c>
+      <c r="I3" s="2">
+        <f>H3^2</f>
+        <v>10.139113857366796</v>
+      </c>
+      <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="F3" s="2">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3">
-        <f>10^(G3/20)</f>
-        <v>1</v>
-      </c>
-      <c r="I3" s="3">
-        <f>H3^2</f>
-        <v>1</v>
-      </c>
-      <c r="K3" s="2">
-        <v>1</v>
-      </c>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3">
+      <c r="L3" s="2">
+        <v>14.359</v>
+      </c>
+      <c r="M3" s="2">
         <f>10^(L3/20)</f>
-        <v>1</v>
-      </c>
-      <c r="N3" s="3">
+        <v>5.2233604937722991</v>
+      </c>
+      <c r="N3" s="2">
         <f>M3^2</f>
-        <v>1</v>
+        <v>27.283494847901196</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3">
+      <c r="B4" s="2">
+        <v>-21.094000000000001</v>
+      </c>
+      <c r="C4" s="2">
         <f t="shared" ref="C4:C10" si="0">10^(B4/20)</f>
-        <v>1</v>
-      </c>
-      <c r="D4" s="3">
+        <v>8.8165769026219087E-2</v>
+      </c>
+      <c r="D4" s="2">
         <f t="shared" ref="D4:D10" si="1">C4^2</f>
-        <v>1</v>
-      </c>
-      <c r="F4" s="2">
+        <v>7.7732028279846131E-3</v>
+      </c>
+      <c r="F4" s="1">
         <v>2</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3">
+      <c r="G4" s="2">
+        <v>-5.0990000000000002</v>
+      </c>
+      <c r="H4" s="2">
         <f t="shared" ref="H4:H10" si="2">10^(G4/20)</f>
-        <v>1</v>
-      </c>
-      <c r="I4" s="3">
+        <v>0.55596826179752568</v>
+      </c>
+      <c r="I4" s="2">
         <f t="shared" ref="I4:I10" si="3">H4^2</f>
-        <v>1</v>
-      </c>
-      <c r="K4" s="2">
+        <v>0.30910070812616203</v>
+      </c>
+      <c r="K4" s="1">
         <v>2</v>
       </c>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3">
+      <c r="L4" s="2">
+        <v>-8.6999999999999994E-2</v>
+      </c>
+      <c r="M4" s="2">
         <f t="shared" ref="M4:M10" si="4">10^(L4/20)</f>
-        <v>1</v>
-      </c>
-      <c r="N4" s="3">
+        <v>0.99003375036727115</v>
+      </c>
+      <c r="N4" s="2">
         <f t="shared" ref="N4:N10" si="5">M4^2</f>
-        <v>1</v>
+        <v>0.9801668268662842</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3">
+      <c r="B5" s="2">
+        <v>-53.954000000000001</v>
+      </c>
+      <c r="C5" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D5" s="3">
+        <v>2.0058571459359471E-3</v>
+      </c>
+      <c r="D5" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F5" s="2">
+        <v>4.0234628899023036E-6</v>
+      </c>
+      <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3">
+      <c r="G5" s="2">
+        <v>-31.981999999999999</v>
+      </c>
+      <c r="H5" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I5" s="3">
+        <v>2.5170972779597824E-2</v>
+      </c>
+      <c r="I5" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K5" s="2">
+        <v>6.3357787067125457E-4</v>
+      </c>
+      <c r="K5" s="1">
         <v>3</v>
       </c>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3">
+      <c r="L5" s="2">
+        <v>-20.283999999999999</v>
+      </c>
+      <c r="M5" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N5" s="3">
+        <v>9.6783205048815962E-2</v>
+      </c>
+      <c r="N5" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>9.3669887795211557E-3</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3">
+      <c r="B6" s="2">
+        <v>-62.375</v>
+      </c>
+      <c r="C6" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D6" s="3">
+        <v>7.6076408192626973E-4</v>
+      </c>
+      <c r="D6" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F6" s="2">
+        <v>5.7876198834912002E-7</v>
+      </c>
+      <c r="F6" s="1">
         <v>4</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3">
+      <c r="G6" s="2">
+        <v>-47.223999999999997</v>
+      </c>
+      <c r="H6" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I6" s="3">
+        <v>4.3531135922963808E-3</v>
+      </c>
+      <c r="I6" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K6" s="2">
+        <v>1.89495979474355E-5</v>
+      </c>
+      <c r="K6" s="1">
         <v>4</v>
       </c>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3">
+      <c r="L6" s="2">
+        <v>-29.524999999999999</v>
+      </c>
+      <c r="M6" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N6" s="3">
+        <v>3.3400271725703846E-2</v>
+      </c>
+      <c r="N6" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>1.1155781513508519E-3</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3">
+      <c r="B7" s="2">
+        <v>-58.167000000000002</v>
+      </c>
+      <c r="C7" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D7" s="3">
+        <v>1.2349517787522469E-3</v>
+      </c>
+      <c r="D7" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F7" s="2">
+        <v>1.5251058958433385E-6</v>
+      </c>
+      <c r="F7" s="1">
         <v>5</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3">
+      <c r="G7" s="2">
+        <v>-41.470999999999997</v>
+      </c>
+      <c r="H7" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I7" s="3">
+        <v>8.4420904315600214E-3</v>
+      </c>
+      <c r="I7" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K7" s="2">
+        <v>7.1268890854637274E-5</v>
+      </c>
+      <c r="K7" s="1">
         <v>5</v>
       </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3">
+      <c r="L7" s="2">
+        <v>-21.821000000000002</v>
+      </c>
+      <c r="M7" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N7" s="3">
+        <v>8.1086769788603449E-2</v>
+      </c>
+      <c r="N7" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>6.5750642347499732E-3</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3">
+      <c r="B8" s="2">
+        <v>-65.164000000000001</v>
+      </c>
+      <c r="C8" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D8" s="3">
+        <v>5.5182325675656512E-4</v>
+      </c>
+      <c r="D8" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F8" s="2">
+        <v>3.0450890669742201E-7</v>
+      </c>
+      <c r="F8" s="1">
         <v>6</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3">
+      <c r="G8" s="2">
+        <v>-49.325000000000003</v>
+      </c>
+      <c r="H8" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I8" s="3">
+        <v>3.4178263997185748E-3</v>
+      </c>
+      <c r="I8" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K8" s="2">
+        <v>1.1681537298613235E-5</v>
+      </c>
+      <c r="K8" s="1">
         <v>6</v>
       </c>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3">
+      <c r="L8" s="2">
+        <v>-33.03</v>
+      </c>
+      <c r="M8" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N8" s="3">
+        <v>2.2310022074819549E-2</v>
+      </c>
+      <c r="N8" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>4.9773708497893561E-4</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3">
+      <c r="B9" s="2">
+        <v>-56.576999999999998</v>
+      </c>
+      <c r="C9" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D9" s="3">
+        <v>1.4830302171893748E-3</v>
+      </c>
+      <c r="D9" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F9" s="2">
+        <v>2.1993786250967641E-6</v>
+      </c>
+      <c r="F9" s="1">
         <v>7</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3">
+      <c r="G9" s="2">
+        <v>-39.351999999999997</v>
+      </c>
+      <c r="H9" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I9" s="3">
+        <v>1.0774571314563667E-2</v>
+      </c>
+      <c r="I9" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K9" s="2">
+        <v>1.1609138701261823E-4</v>
+      </c>
+      <c r="K9" s="1">
         <v>7</v>
       </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3">
+      <c r="L9" s="2">
+        <v>-25.943000000000001</v>
+      </c>
+      <c r="M9" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N9" s="3">
+        <v>5.0448702382415216E-2</v>
+      </c>
+      <c r="N9" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>2.5450715720695067E-3</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3">
+      <c r="B10" s="2">
+        <v>-69.899000000000001</v>
+      </c>
+      <c r="C10" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D10" s="3">
+        <v>3.199263417302159E-4</v>
+      </c>
+      <c r="D10" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F10" s="2">
+        <v>1.0235286413287889E-7</v>
+      </c>
+      <c r="F10" s="1">
         <v>8</v>
       </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3">
+      <c r="G10" s="2">
+        <v>-45.615000000000002</v>
+      </c>
+      <c r="H10" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I10" s="3">
+        <v>5.2390193199477039E-3</v>
+      </c>
+      <c r="I10" s="2">
         <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="K10" s="2">
+        <v>2.7447323434785302E-5</v>
+      </c>
+      <c r="K10" s="1">
         <v>8</v>
       </c>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3">
+      <c r="L10" s="2">
+        <v>-43.009</v>
+      </c>
+      <c r="M10" s="2">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="N10" s="3">
+        <v>7.0721261685597614E-3</v>
+      </c>
+      <c r="N10" s="2">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>5.0014968544027768E-5</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <f>SQRT(SUM(D4:D10)/D3)</f>
-        <v>2.6457513110645907</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="F11" s="2" t="s">
+        <v>0.17589108930319319</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="F11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="2">
         <f>SQRT(SUM(I4:I10)/I3)</f>
-        <v>2.6457513110645907</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="K11" s="2" t="s">
+        <v>0.174850405623248</v>
+      </c>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="K11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="2">
         <f>SQRT(SUM(N4:N10)/N3)</f>
-        <v>2.6457513110645907</v>
-      </c>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
+        <v>0.19147800145897581</v>
+      </c>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <f>B11*100</f>
-        <v>264.57513110645908</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="F12" s="4" t="s">
+        <v>17.58910893031932</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="F12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <f>G11*100</f>
-        <v>264.57513110645908</v>
-      </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="K12" s="4" t="s">
+        <v>17.485040562324798</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="K12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L12" s="4">
         <f>L11*100</f>
-        <v>264.57513110645908</v>
-      </c>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
+        <v>19.14780014589758</v>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="2">
-        <f>(B16^2/250) * 1000</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="F13" s="2" t="s">
+      <c r="B13" s="1">
+        <v>2.5920000000000001</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="F13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="2">
-        <f>(G16^2/250) * 1000</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="K13" s="2" t="s">
+      <c r="G13" s="1">
+        <v>105.8</v>
+      </c>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="K13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L13" s="2">
-        <f>(L16^2/250) * 1000</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
+      <c r="L13" s="1">
+        <v>211.25</v>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="2">
-        <v>116.68</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="F14" s="2" t="s">
+      <c r="B14" s="1">
+        <v>68.277000000000001</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="F14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G14" s="2">
-        <v>116.68</v>
-      </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="K14" s="2" t="s">
+      <c r="G14" s="1">
+        <v>372.423</v>
+      </c>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="K14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L14" s="2">
-        <v>116.68</v>
-      </c>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
+      <c r="L14" s="1">
+        <v>620.70399999999995</v>
+      </c>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <f>(B13/B14)*100</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="F15" s="4" t="s">
+        <v>3.7963003646908917</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="F15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <f>(G13/G14)*100</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="K15" s="4" t="s">
+        <v>28.408556936601659</v>
+      </c>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="K15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L15" s="4">
+      <c r="L15" s="3">
         <f>(L13/L14)*100</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
+        <v>34.033935660153638</v>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>